<commit_message>
Preenche custo e preço de venda dos 37 itens; atualiza planilha
Custo e preço de venda foram gravados no banco ao vivo (37 writes) e
refletidos na planilha, que agora calcula o valor total do estoque a
preço de custo: R$ 120.348,50.

9403 STD, 2900 e 8566 STD ficaram só com custo (sem preço de venda na
lista recebida).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165A6Br55Xm9UacbZKzKy8q
</commit_message>
<xml_diff>
--- a/dados/estoque-2026-09-25.xlsx
+++ b/dados/estoque-2026-09-25.xlsx
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -634,11 +634,11 @@
       </c>
       <c r="B6" s="6">
         <f>SUM(Estoque!I2:I38)</f>
-        <v>0</v>
+        <v>120348.5</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Só preenche depois que você informar o custo unitário.</t>
+          <t>Valor total do estoque, a preço de custo.</t>
         </is>
       </c>
     </row>
@@ -748,58 +748,50 @@
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>• As células amarelas da aba Estoque são as que você preenche: Estoque mínimo, Custo unit. e Preço venda.</t>
+          <t>• As células amarelas da aba Estoque (mínimo, custo e preço de venda) já vêm preenchidas — edite direto ali se algum valor mudar.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>• Formato esperado nessas colunas: número puro, sem R$ e sem ponto de milhar. Ex.: mínimo 50 · custo 12,90 · preço 27,50.</t>
+          <t>• Formato dessas colunas: número puro, sem R$ e sem ponto de milhar. Ex.: mínimo 50 · custo 12,90 · preço 27,50.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>• Preenchendo o mínimo, a coluna Situação passa a marcar "Abaixo do mínimo" sozinha.</t>
+          <t>• 9403 STD, 2900 e 8566 STD ainda estão sem preço de venda informado — só o custo.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>• Preenchendo o custo, as colunas Valor em custo e o total do Resumo se calculam sozinhos.</t>
+          <t>• As colunas Valor em custo, Situação e Vendido (histórico) são fórmulas — não digite nada nelas.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>• As colunas Valor em custo, Situação e Vendido (histórico) são fórmulas — não digite nada nelas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
           <t>• Esta planilha é uma foto do dia 25/09. O saldo que vale é o do app, que atualiza na hora.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>App do estoque: https://claude.ai/artifact/JiMT1jfH7Vc3MUYtYcDNG7</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A16:C16"/>
   </mergeCells>
@@ -911,11 +903,15 @@
         <v>289</v>
       </c>
       <c r="F2" s="13" t="n"/>
-      <c r="G2" s="14" t="n"/>
-      <c r="H2" s="14" t="n"/>
+      <c r="G2" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="H2" s="14" t="n">
+        <v>142.25</v>
+      </c>
       <c r="I2" s="15">
         <f>E2*G2</f>
-        <v>0</v>
+        <v>21675</v>
       </c>
       <c t="str" r="J2" s="11">
         <f>IF(E2&lt;0,"Negativo",IF(E2=0,"Sem estoque",IF(AND(F2&gt;0,E2&lt;=F2),"Abaixo do mínimo","OK")))</f>
@@ -951,11 +947,15 @@
         <v>99</v>
       </c>
       <c r="F3" s="13" t="n"/>
-      <c r="G3" s="14" t="n"/>
-      <c r="H3" s="14" t="n"/>
+      <c r="G3" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="H3" s="14" t="n">
+        <v>148.56</v>
+      </c>
       <c r="I3" s="15">
         <f>E3*G3</f>
-        <v>0</v>
+        <v>7425</v>
       </c>
       <c t="str" r="J3" s="11">
         <f>IF(E3&lt;0,"Negativo",IF(E3=0,"Sem estoque",IF(AND(F3&gt;0,E3&lt;=F3),"Abaixo do mínimo","OK")))</f>
@@ -991,11 +991,15 @@
         <v>22</v>
       </c>
       <c r="F4" s="13" t="n"/>
-      <c r="G4" s="14" t="n"/>
-      <c r="H4" s="14" t="n"/>
+      <c r="G4" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>127.94</v>
+      </c>
       <c r="I4" s="15">
         <f>E4*G4</f>
-        <v>0</v>
+        <v>1650</v>
       </c>
       <c t="str" r="J4" s="11">
         <f>IF(E4&lt;0,"Negativo",IF(E4=0,"Sem estoque",IF(AND(F4&gt;0,E4&lt;=F4),"Abaixo do mínimo","OK")))</f>
@@ -1031,11 +1035,15 @@
         <v>1</v>
       </c>
       <c r="F5" s="13" t="n"/>
-      <c r="G5" s="14" t="n"/>
-      <c r="H5" s="14" t="n"/>
+      <c r="G5" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>144.9</v>
+      </c>
       <c r="I5" s="15">
         <f>E5*G5</f>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c t="str" r="J5" s="11">
         <f>IF(E5&lt;0,"Negativo",IF(E5=0,"Sem estoque",IF(AND(F5&gt;0,E5&lt;=F5),"Abaixo do mínimo","OK")))</f>
@@ -1071,11 +1079,15 @@
         <v>7</v>
       </c>
       <c r="F6" s="13" t="n"/>
-      <c r="G6" s="14" t="n"/>
-      <c r="H6" s="14" t="n"/>
+      <c r="G6" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="H6" s="14" t="n">
+        <v>156.03</v>
+      </c>
       <c r="I6" s="15">
         <f>E6*G6</f>
-        <v>0</v>
+        <v>525</v>
       </c>
       <c t="str" r="J6" s="11">
         <f>IF(E6&lt;0,"Negativo",IF(E6=0,"Sem estoque",IF(AND(F6&gt;0,E6&lt;=F6),"Abaixo do mínimo","OK")))</f>
@@ -1111,11 +1123,13 @@
         <v>20</v>
       </c>
       <c r="F7" s="13" t="n"/>
-      <c r="G7" s="14" t="n"/>
+      <c r="G7" s="14" t="n">
+        <v>75</v>
+      </c>
       <c r="H7" s="14" t="n"/>
       <c r="I7" s="15">
         <f>E7*G7</f>
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c t="str" r="J7" s="11">
         <f>IF(E7&lt;0,"Negativo",IF(E7=0,"Sem estoque",IF(AND(F7&gt;0,E7&lt;=F7),"Abaixo do mínimo","OK")))</f>
@@ -1151,11 +1165,15 @@
         <v>22</v>
       </c>
       <c r="F8" s="13" t="n"/>
-      <c r="G8" s="14" t="n"/>
-      <c r="H8" s="14" t="n"/>
+      <c r="G8" s="14" t="n">
+        <v>32</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>69.25</v>
+      </c>
       <c r="I8" s="15">
         <f>E8*G8</f>
-        <v>0</v>
+        <v>704</v>
       </c>
       <c t="str" r="J8" s="11">
         <f>IF(E8&lt;0,"Negativo",IF(E8=0,"Sem estoque",IF(AND(F8&gt;0,E8&lt;=F8),"Abaixo do mínimo","OK")))</f>
@@ -1191,11 +1209,15 @@
         <v>51</v>
       </c>
       <c r="F9" s="13" t="n"/>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="n"/>
+      <c r="G9" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>172.55</v>
+      </c>
       <c r="I9" s="15">
         <f>E9*G9</f>
-        <v>0</v>
+        <v>3825</v>
       </c>
       <c t="str" r="J9" s="11">
         <f>IF(E9&lt;0,"Negativo",IF(E9=0,"Sem estoque",IF(AND(F9&gt;0,E9&lt;=F9),"Abaixo do mínimo","OK")))</f>
@@ -1231,11 +1253,15 @@
         <v>35</v>
       </c>
       <c r="F10" s="13" t="n"/>
-      <c r="G10" s="14" t="n"/>
-      <c r="H10" s="14" t="n"/>
+      <c r="G10" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="H10" s="14" t="n">
+        <v>126.81</v>
+      </c>
       <c r="I10" s="15">
         <f>E10*G10</f>
-        <v>0</v>
+        <v>2625</v>
       </c>
       <c t="str" r="J10" s="11">
         <f>IF(E10&lt;0,"Negativo",IF(E10=0,"Sem estoque",IF(AND(F10&gt;0,E10&lt;=F10),"Abaixo do mínimo","OK")))</f>
@@ -1271,11 +1297,15 @@
         <v>116</v>
       </c>
       <c r="F11" s="13" t="n"/>
-      <c r="G11" s="14" t="n"/>
-      <c r="H11" s="14" t="n"/>
+      <c r="G11" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="H11" s="14" t="n">
+        <v>31.13</v>
+      </c>
       <c r="I11" s="15">
         <f>E11*G11</f>
-        <v>0</v>
+        <v>1392</v>
       </c>
       <c t="str" r="J11" s="11">
         <f>IF(E11&lt;0,"Negativo",IF(E11=0,"Sem estoque",IF(AND(F11&gt;0,E11&lt;=F11),"Abaixo do mínimo","OK")))</f>
@@ -1311,11 +1341,15 @@
         <v>558</v>
       </c>
       <c r="F12" s="13" t="n"/>
-      <c r="G12" s="14" t="n"/>
-      <c r="H12" s="14" t="n"/>
+      <c r="G12" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>12.32</v>
+      </c>
       <c r="I12" s="15">
         <f>E12*G12</f>
-        <v>0</v>
+        <v>4464</v>
       </c>
       <c t="str" r="J12" s="11">
         <f>IF(E12&lt;0,"Negativo",IF(E12=0,"Sem estoque",IF(AND(F12&gt;0,E12&lt;=F12),"Abaixo do mínimo","OK")))</f>
@@ -1351,11 +1385,15 @@
         <v>124</v>
       </c>
       <c r="F13" s="13" t="n"/>
-      <c r="G13" s="14" t="n"/>
-      <c r="H13" s="14" t="n"/>
+      <c r="G13" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>13.42</v>
+      </c>
       <c r="I13" s="15">
         <f>E13*G13</f>
-        <v>0</v>
+        <v>992</v>
       </c>
       <c t="str" r="J13" s="11">
         <f>IF(E13&lt;0,"Negativo",IF(E13=0,"Sem estoque",IF(AND(F13&gt;0,E13&lt;=F13),"Abaixo do mínimo","OK")))</f>
@@ -1391,11 +1429,15 @@
         <v>311</v>
       </c>
       <c r="F14" s="13" t="n"/>
-      <c r="G14" s="14" t="n"/>
-      <c r="H14" s="14" t="n"/>
+      <c r="G14" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" s="14" t="n">
+        <v>11.18</v>
+      </c>
       <c r="I14" s="15">
         <f>E14*G14</f>
-        <v>0</v>
+        <v>2488</v>
       </c>
       <c t="str" r="J14" s="11">
         <f>IF(E14&lt;0,"Negativo",IF(E14=0,"Sem estoque",IF(AND(F14&gt;0,E14&lt;=F14),"Abaixo do mínimo","OK")))</f>
@@ -1431,11 +1473,15 @@
         <v>268</v>
       </c>
       <c r="F15" s="13" t="n"/>
-      <c r="G15" s="14" t="n"/>
-      <c r="H15" s="14" t="n"/>
+      <c r="G15" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="H15" s="14" t="n">
+        <v>28.18</v>
+      </c>
       <c r="I15" s="15">
         <f>E15*G15</f>
-        <v>0</v>
+        <v>4020</v>
       </c>
       <c t="str" r="J15" s="11">
         <f>IF(E15&lt;0,"Negativo",IF(E15=0,"Sem estoque",IF(AND(F15&gt;0,E15&lt;=F15),"Abaixo do mínimo","OK")))</f>
@@ -1471,11 +1517,15 @@
         <v>72</v>
       </c>
       <c r="F16" s="13" t="n"/>
-      <c r="G16" s="14" t="n"/>
-      <c r="H16" s="14" t="n"/>
+      <c r="G16" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>25.62</v>
+      </c>
       <c r="I16" s="15">
         <f>E16*G16</f>
-        <v>0</v>
+        <v>576</v>
       </c>
       <c t="str" r="J16" s="11">
         <f>IF(E16&lt;0,"Negativo",IF(E16=0,"Sem estoque",IF(AND(F16&gt;0,E16&lt;=F16),"Abaixo do mínimo","OK")))</f>
@@ -1511,11 +1561,15 @@
         <v>434</v>
       </c>
       <c r="F17" s="13" t="n"/>
-      <c r="G17" s="14" t="n"/>
-      <c r="H17" s="14" t="n"/>
+      <c r="G17" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H17" s="14" t="n">
+        <v>10.3</v>
+      </c>
       <c r="I17" s="15">
         <f>E17*G17</f>
-        <v>0</v>
+        <v>3038</v>
       </c>
       <c t="str" r="J17" s="11">
         <f>IF(E17&lt;0,"Negativo",IF(E17=0,"Sem estoque",IF(AND(F17&gt;0,E17&lt;=F17),"Abaixo do mínimo","OK")))</f>
@@ -1551,11 +1605,15 @@
         <v>359</v>
       </c>
       <c r="F18" s="13" t="n"/>
-      <c r="G18" s="14" t="n"/>
-      <c r="H18" s="14" t="n"/>
+      <c r="G18" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H18" s="14" t="n">
+        <v>20</v>
+      </c>
       <c r="I18" s="15">
         <f>E18*G18</f>
-        <v>0</v>
+        <v>2513</v>
       </c>
       <c t="str" r="J18" s="11">
         <f>IF(E18&lt;0,"Negativo",IF(E18=0,"Sem estoque",IF(AND(F18&gt;0,E18&lt;=F18),"Abaixo do mínimo","OK")))</f>
@@ -1591,11 +1649,15 @@
         <v>94</v>
       </c>
       <c r="F19" s="13" t="n"/>
-      <c r="G19" s="14" t="n"/>
-      <c r="H19" s="14" t="n"/>
+      <c r="G19" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H19" s="14" t="n">
+        <v>22.16</v>
+      </c>
       <c r="I19" s="15">
         <f>E19*G19</f>
-        <v>0</v>
+        <v>564</v>
       </c>
       <c t="str" r="J19" s="11">
         <f>IF(E19&lt;0,"Negativo",IF(E19=0,"Sem estoque",IF(AND(F19&gt;0,E19&lt;=F19),"Abaixo do mínimo","OK")))</f>
@@ -1631,11 +1693,15 @@
         <v>297</v>
       </c>
       <c r="F20" s="13" t="n"/>
-      <c r="G20" s="14" t="n"/>
-      <c r="H20" s="14" t="n"/>
+      <c r="G20" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>16.89</v>
+      </c>
       <c r="I20" s="15">
         <f>E20*G20</f>
-        <v>0</v>
+        <v>2376</v>
       </c>
       <c t="str" r="J20" s="11">
         <f>IF(E20&lt;0,"Negativo",IF(E20=0,"Sem estoque",IF(AND(F20&gt;0,E20&lt;=F20),"Abaixo do mínimo","OK")))</f>
@@ -1671,11 +1737,15 @@
         <v>101</v>
       </c>
       <c r="F21" s="13" t="n"/>
-      <c r="G21" s="14" t="n"/>
-      <c r="H21" s="14" t="n"/>
+      <c r="G21" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="H21" s="14" t="n">
+        <v>29.43</v>
+      </c>
       <c r="I21" s="15">
         <f>E21*G21</f>
-        <v>0</v>
+        <v>1414</v>
       </c>
       <c t="str" r="J21" s="11">
         <f>IF(E21&lt;0,"Negativo",IF(E21=0,"Sem estoque",IF(AND(F21&gt;0,E21&lt;=F21),"Abaixo do mínimo","OK")))</f>
@@ -1711,11 +1781,15 @@
         <v>599</v>
       </c>
       <c r="F22" s="13" t="n"/>
-      <c r="G22" s="14" t="n"/>
-      <c r="H22" s="14" t="n"/>
+      <c r="G22" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H22" s="14" t="n">
+        <v>13.23</v>
+      </c>
       <c r="I22" s="15">
         <f>E22*G22</f>
-        <v>0</v>
+        <v>4792</v>
       </c>
       <c t="str" r="J22" s="11">
         <f>IF(E22&lt;0,"Negativo",IF(E22=0,"Sem estoque",IF(AND(F22&gt;0,E22&lt;=F22),"Abaixo do mínimo","OK")))</f>
@@ -1751,11 +1825,15 @@
         <v>35</v>
       </c>
       <c r="F23" s="13" t="n"/>
-      <c r="G23" s="14" t="n"/>
-      <c r="H23" s="14" t="n"/>
+      <c r="G23" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H23" s="14" t="n">
+        <v>21.5</v>
+      </c>
       <c r="I23" s="15">
         <f>E23*G23</f>
-        <v>0</v>
+        <v>280</v>
       </c>
       <c t="str" r="J23" s="11">
         <f>IF(E23&lt;0,"Negativo",IF(E23=0,"Sem estoque",IF(AND(F23&gt;0,E23&lt;=F23),"Abaixo do mínimo","OK")))</f>
@@ -1791,11 +1869,15 @@
         <v>211</v>
       </c>
       <c r="F24" s="13" t="n"/>
-      <c r="G24" s="14" t="n"/>
-      <c r="H24" s="14" t="n"/>
+      <c r="G24" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>18.31</v>
+      </c>
       <c r="I24" s="15">
         <f>E24*G24</f>
-        <v>0</v>
+        <v>2532</v>
       </c>
       <c t="str" r="J24" s="11">
         <f>IF(E24&lt;0,"Negativo",IF(E24=0,"Sem estoque",IF(AND(F24&gt;0,E24&lt;=F24),"Abaixo do mínimo","OK")))</f>
@@ -1831,11 +1913,15 @@
         <v>483</v>
       </c>
       <c r="F25" s="13" t="n"/>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="14" t="n"/>
+      <c r="G25" s="14" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>13.38</v>
+      </c>
       <c r="I25" s="15">
         <f>E25*G25</f>
-        <v>0</v>
+        <v>4105.5</v>
       </c>
       <c t="str" r="J25" s="11">
         <f>IF(E25&lt;0,"Negativo",IF(E25=0,"Sem estoque",IF(AND(F25&gt;0,E25&lt;=F25),"Abaixo do mínimo","OK")))</f>
@@ -1871,11 +1957,15 @@
         <v>892</v>
       </c>
       <c r="F26" s="13" t="n"/>
-      <c r="G26" s="14" t="n"/>
-      <c r="H26" s="14" t="n"/>
+      <c r="G26" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H26" s="14" t="n">
+        <v>13.36</v>
+      </c>
       <c r="I26" s="15">
         <f>E26*G26</f>
-        <v>0</v>
+        <v>7136</v>
       </c>
       <c t="str" r="J26" s="11">
         <f>IF(E26&lt;0,"Negativo",IF(E26=0,"Sem estoque",IF(AND(F26&gt;0,E26&lt;=F26),"Abaixo do mínimo","OK")))</f>
@@ -1911,11 +2001,15 @@
         <v>50</v>
       </c>
       <c r="F27" s="13" t="n"/>
-      <c r="G27" s="14" t="n"/>
-      <c r="H27" s="14" t="n"/>
+      <c r="G27" s="14" t="n">
+        <v>55</v>
+      </c>
+      <c r="H27" s="14" t="n">
+        <v>68.34999999999999</v>
+      </c>
       <c r="I27" s="15">
         <f>E27*G27</f>
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c t="str" r="J27" s="11">
         <f>IF(E27&lt;0,"Negativo",IF(E27=0,"Sem estoque",IF(AND(F27&gt;0,E27&lt;=F27),"Abaixo do mínimo","OK")))</f>
@@ -1951,11 +2045,15 @@
         <v>15</v>
       </c>
       <c r="F28" s="13" t="n"/>
-      <c r="G28" s="14" t="n"/>
-      <c r="H28" s="14" t="n"/>
+      <c r="G28" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>25.62</v>
+      </c>
       <c r="I28" s="15">
         <f>E28*G28</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c t="str" r="J28" s="11">
         <f>IF(E28&lt;0,"Negativo",IF(E28=0,"Sem estoque",IF(AND(F28&gt;0,E28&lt;=F28),"Abaixo do mínimo","OK")))</f>
@@ -1991,11 +2089,15 @@
         <v>122</v>
       </c>
       <c r="F29" s="13" t="n"/>
-      <c r="G29" s="14" t="n"/>
-      <c r="H29" s="14" t="n"/>
+      <c r="G29" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="H29" s="14" t="n">
+        <v>88.68000000000001</v>
+      </c>
       <c r="I29" s="15">
         <f>E29*G29</f>
-        <v>0</v>
+        <v>7320</v>
       </c>
       <c t="str" r="J29" s="11">
         <f>IF(E29&lt;0,"Negativo",IF(E29=0,"Sem estoque",IF(AND(F29&gt;0,E29&lt;=F29),"Abaixo do mínimo","OK")))</f>
@@ -2031,11 +2133,15 @@
         <v>44</v>
       </c>
       <c r="F30" s="13" t="n"/>
-      <c r="G30" s="14" t="n"/>
-      <c r="H30" s="14" t="n"/>
+      <c r="G30" s="14" t="n">
+        <v>70</v>
+      </c>
+      <c r="H30" s="14" t="n">
+        <v>119.3</v>
+      </c>
       <c r="I30" s="15">
         <f>E30*G30</f>
-        <v>0</v>
+        <v>3080</v>
       </c>
       <c t="str" r="J30" s="11">
         <f>IF(E30&lt;0,"Negativo",IF(E30=0,"Sem estoque",IF(AND(F30&gt;0,E30&lt;=F30),"Abaixo do mínimo","OK")))</f>
@@ -2071,11 +2177,15 @@
         <v>148</v>
       </c>
       <c r="F31" s="13" t="n"/>
-      <c r="G31" s="14" t="n"/>
-      <c r="H31" s="14" t="n"/>
+      <c r="G31" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="H31" s="14" t="n">
+        <v>38.88</v>
+      </c>
       <c r="I31" s="15">
         <f>E31*G31</f>
-        <v>0</v>
+        <v>3700</v>
       </c>
       <c t="str" r="J31" s="11">
         <f>IF(E31&lt;0,"Negativo",IF(E31=0,"Sem estoque",IF(AND(F31&gt;0,E31&lt;=F31),"Abaixo do mínimo","OK")))</f>
@@ -2111,11 +2221,15 @@
         <v>27</v>
       </c>
       <c r="F32" s="13" t="n"/>
-      <c r="G32" s="14" t="n"/>
-      <c r="H32" s="14" t="n"/>
+      <c r="G32" s="14" t="n">
+        <v>95</v>
+      </c>
+      <c r="H32" s="14" t="n">
+        <v>231.86</v>
+      </c>
       <c r="I32" s="15">
         <f>E32*G32</f>
-        <v>0</v>
+        <v>2565</v>
       </c>
       <c t="str" r="J32" s="11">
         <f>IF(E32&lt;0,"Negativo",IF(E32=0,"Sem estoque",IF(AND(F32&gt;0,E32&lt;=F32),"Abaixo do mínimo","OK")))</f>
@@ -2151,11 +2265,15 @@
         <v>3</v>
       </c>
       <c r="F33" s="13" t="n"/>
-      <c r="G33" s="14" t="n"/>
-      <c r="H33" s="14" t="n"/>
+      <c r="G33" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="H33" s="14" t="n">
+        <v>57.36</v>
+      </c>
       <c r="I33" s="15">
         <f>E33*G33</f>
-        <v>0</v>
+        <v>150</v>
       </c>
       <c t="str" r="J33" s="11">
         <f>IF(E33&lt;0,"Negativo",IF(E33=0,"Sem estoque",IF(AND(F33&gt;0,E33&lt;=F33),"Abaixo do mínimo","OK")))</f>
@@ -2191,11 +2309,15 @@
         <v>148</v>
       </c>
       <c r="F34" s="13" t="n"/>
-      <c r="G34" s="14" t="n"/>
-      <c r="H34" s="14" t="n"/>
+      <c r="G34" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="H34" s="14" t="n">
+        <v>70.29000000000001</v>
+      </c>
       <c r="I34" s="15">
         <f>E34*G34</f>
-        <v>0</v>
+        <v>7400</v>
       </c>
       <c t="str" r="J34" s="11">
         <f>IF(E34&lt;0,"Negativo",IF(E34=0,"Sem estoque",IF(AND(F34&gt;0,E34&lt;=F34),"Abaixo do mínimo","OK")))</f>
@@ -2231,11 +2353,15 @@
         <v>29</v>
       </c>
       <c r="F35" s="13" t="n"/>
-      <c r="G35" s="14" t="n"/>
-      <c r="H35" s="14" t="n"/>
+      <c r="G35" s="14" t="n">
+        <v>85</v>
+      </c>
+      <c r="H35" s="14" t="n">
+        <v>145.76</v>
+      </c>
       <c r="I35" s="15">
         <f>E35*G35</f>
-        <v>0</v>
+        <v>2465</v>
       </c>
       <c t="str" r="J35" s="11">
         <f>IF(E35&lt;0,"Negativo",IF(E35=0,"Sem estoque",IF(AND(F35&gt;0,E35&lt;=F35),"Abaixo do mínimo","OK")))</f>
@@ -2271,11 +2397,15 @@
         <v>318</v>
       </c>
       <c r="F36" s="13" t="n"/>
-      <c r="G36" s="14" t="n"/>
-      <c r="H36" s="14" t="n"/>
+      <c r="G36" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="H36" s="14" t="n">
+        <v>13.36</v>
+      </c>
       <c r="I36" s="15">
         <f>E36*G36</f>
-        <v>0</v>
+        <v>2862</v>
       </c>
       <c t="str" r="J36" s="11">
         <f>IF(E36&lt;0,"Negativo",IF(E36=0,"Sem estoque",IF(AND(F36&gt;0,E36&lt;=F36),"Abaixo do mínimo","OK")))</f>
@@ -2307,11 +2437,13 @@
         <v>50</v>
       </c>
       <c r="F37" s="13" t="n"/>
-      <c r="G37" s="14" t="n"/>
+      <c r="G37" s="14" t="n">
+        <v>75</v>
+      </c>
       <c r="H37" s="14" t="n"/>
       <c r="I37" s="15">
         <f>E37*G37</f>
-        <v>0</v>
+        <v>3750</v>
       </c>
       <c t="str" r="J37" s="11">
         <f>IF(E37&lt;0,"Negativo",IF(E37=0,"Sem estoque",IF(AND(F37&gt;0,E37&lt;=F37),"Abaixo do mínimo","OK")))</f>
@@ -2343,11 +2475,13 @@
         <v>20</v>
       </c>
       <c r="F38" s="13" t="n"/>
-      <c r="G38" s="14" t="n"/>
+      <c r="G38" s="14" t="n">
+        <v>75</v>
+      </c>
       <c r="H38" s="14" t="n"/>
       <c r="I38" s="15">
         <f>E38*G38</f>
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c t="str" r="J38" s="11">
         <f>IF(E38&lt;0,"Negativo",IF(E38=0,"Sem estoque",IF(AND(F38&gt;0,E38&lt;=F38),"Abaixo do mínimo","OK")))</f>
@@ -2370,7 +2504,7 @@
       </c>
       <c r="I39" s="18">
         <f>SUM(I2:I38)</f>
-        <v>0</v>
+        <v>120348.5</v>
       </c>
       <c r="K39" s="17">
         <f>SUM(K2:K38)</f>

</xml_diff>